<commit_message>
feat(opd): add OPD test cases T16-T25 (Quantity, Approval, Doctor, Price, Discount, Favorites 'اليكو 2026', Medicines Tab, Credit Pct) and update Excel doc
</commit_message>
<xml_diff>
--- a/Paymax Automation Test Cases-Aug16-2026.xlsx
+++ b/Paymax Automation Test Cases-Aug16-2026.xlsx
@@ -556,9 +556,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -892,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4784,6 +4782,726 @@
       <c r="N55" s="7" t="inlineStr">
         <is>
           <t>Added 2026-08-16 — Complete OPD service draft &amp; save cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TC-OPD-019</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Service quantity field rules (min 1; locked for non-countable vs custom for countable)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>قواعد حقل العدد للخدمة (يجب أن يكون &gt;= 1؛ مغلق للخدمات غير القابلة للعد ومفتوح للخدمات القابلة للعد)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Verify that quantity defaults to 1 and is locked for non-countable service ('خدمة الظهر الشاملة الكاملة 1'), while countable service ('مفاصل الظهر') allows entering custom quantity.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>التحقق من أن العدد يبدأ بـ 1 ويكون مغلقاً للخدمة غير القابلة للعد، ومفتوحاً لإدخال العدد للخدمة القابلة للعد.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>verifyServiceQuantityFieldRules</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Service quantity rules (non-countable vs countable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>TC-OPD-020</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Approval number mandatory validation rules</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>قواعد إجبارية رقم الموافقة للخدمات التي تتطلب موافقة</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Verify that adding a service requiring approval number without entering approval number displays validation error 'برجاء إدخال رقم الموافقة', while service not requiring approval does not mandate it.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>التحقق من أن إضافة خدمة تطلب موافقة بدون إدخال رقم الموافقة يظهر رسالة تحذير، بينما الخدمة التي لا تطلب موافقة لا تشترط ذلك.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>verifyApprovalNumberRules</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Approval number mandatory validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>TC-OPD-021</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Doctor selection mandatory rules by service configuration</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>قواعد إجبارية الطبيب حسب إعدادات الخدمة</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Verify adding service not requiring doctor ('كشف ظهر كامل') succeeds without doctor, while service requiring doctor ('كشف ظهر') displays doctor selection validation error.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>التحقق من أن الخدمة التي لا تطلب طبيباً تنزل للقائمة بدون طبيب، بينما الخدمة التي تتطلب طبيباً تظهر رسالة خطأ عند عدم اختياره.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>verifyDoctorMandatoryRules</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Doctor mandatory validation rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TC-OPD-022</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Service unit price editability rules (fixed vs editable)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>قواعد تعديل سعر وحدة الخدمة (سعر ثابت مغلق مقابل سعر قابل للتعديل)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Verify price field is locked/readonly for fixed-price service ('خدمة الظهر الشاملة الكاملة 1') and editable for variable-price service.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>التحقق من أن سعر الخدمة الثابتة يكون مغلقاً ومحدداً مسبقاً، وسعر الخدمة القابلة للتعديل يكون مفتوحاً للكتابة.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>verifyServicePriceEditableRules</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Fixed price vs editable price rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TC-OPD-023</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Discount giver mandatory rules when discount percentage is applied</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>قواعد مانح الخصم عند إدخال نسبة خصم على الخدمة</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Verify discount giver DDL is disabled by default, opens when discount % is entered, and mandates selecting discount giver before adding service.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>التحقق من أن مانح الخصم يكون مغلقاً افتراضياً ويفتح عند إدخال نسبة خصم، وتشترط الصفحة اختياره قبل إضافة الخدمة.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>verifyDiscountGiverMandatoryRules</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Discount giver mandatory validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TC-OPD-024</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Discount percentage upper limit (&gt;100%) and negative value validation</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>حدود نسبة الخصم (عدم تجاوز 100% والرفض للقيم السالبة)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Verify entering discount &gt; 100% displays error 'نسبة الخصم يجب ألا تزيد عن 100%' and clears field, and negative % displays validation error.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>التحقق من إظهار تنبيه عند إدخال نسبة خصم أكبر من 100% وتفريغ الفيلد، وإظهار خطأ عند إدخال قيمة سالبة.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>verifyDiscountPercentageLimits</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Discount percentage range validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TC-OPD-025</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Favorites list toggle, favorite menu selection ('اليكو 2026') and item checkboxes</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>إظهار قائمة المفضلة واختيار قائمة 'اليكو 2026' وظهور خيارات الخدمات والأشعة والتحاليل</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Verify clicking 'إظهار المفضلة' opens favorite menu dropdown, selecting favorite menu 'اليكو 2026' displays favorite item checkboxes.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>التحقق من أن زرار 'إظهار المفضلة' يفتح DDL القوائم المفضلة، واختيار قائمة 'اليكو 2026' يظهر عناصر الـ Checkboxes الخاصة بالخدمات والأشعة والتحاليل.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>favoritesListToggleAndItemSelection</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Favorites list &amp; favorite menu اليكو 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TC-OPD-026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Medicines tab initial empty state for Store/Doctor and '+' batch button toggle</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>الحالة الأولى لتاب صرف الأدوية (اختر المخزن، اختر الطبيب) وظهور علامة الـ + بعد اختيار المخزن والطبيب</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Verify store and doctor DDLs default to 'اختر المخزن' and 'اختر الطبيب', '+' button is hidden initially and becomes visible after selecting store 'main store' and doctor 'Ahmed Badawi'.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>التحقق من أن DDL المخزن والطبيب يبدءان بدون اختيار، وعلامة الـ + لا تظهر إلا بعد اختيار مخزن 'main store' والطبيب 'Ahmed Badawi'.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>medicinesTabInitialStateAndStoreDoctorSelection</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Medicines tab initial state &amp; store/doctor selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TC-OPD-027</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Medicines tab item &amp; unit selection, batch dialog '+', and 'جديد' clear button</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>اختيار صنف 'يورانيوم مشع' والوحدة 'حبيبات' وعلامة الـ + وزرار 'جديد' لتفريغ البيانات</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Select item 'يورانيوم مشع', unit 'حبيبات', click '+' batch button, click 'جديد' (clear button) and verify store, doctor, and item selections are cleared.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>اختيار صنف 'يورانيوم مشع' والوحدة 'حبيبات' والضغط على علامة الـ + ثم الضغط على 'جديد' والتأكد من تفريغ داتا المخزن والطبيب والأصناف.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>medicinesTabItemSelectionBatchAndClearData</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Medicines tab item, unit, batch dialog &amp; clear button</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TC-OPD-028</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Medicines tab credit percentage field (نسبة التحمل) validation for Cash vs Credit entities</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>فيلد نسبة التحمل في تاب صرف الأدوية (مغلق للجهات النقدي ومفتوح للجهات الآجل من 0 لـ 100%)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Verify credit percentage field is locked/readonly for cash entity visits and open/editable (0-100%) for credit entity visits ('اليكو').</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>التحقق من أن فيلد نسبة التحمل يكون مغلقاً في حالة جهة المريض نقدي، ومفتوحاً ويقبل نسب من 0 إلى 100% في حالة جهة المريض آجل.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>medicinesTabCreditPctFieldValidationCashVsCredit</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Medicines tab credit percentage field cash vs credit validation</t>
         </is>
       </c>
     </row>
@@ -4889,10 +5607,10 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(opd): split credit pct test into independent TestNG methods (Cash vs Credit) and improve Angular router navigation back to reception
</commit_message>
<xml_diff>
--- a/Paymax Automation Test Cases-Aug16-2026.xlsx
+++ b/Paymax Automation Test Cases-Aug16-2026.xlsx
@@ -556,7 +556,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -890,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5451,22 +5450,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Medicines tab credit percentage field (نسبة التحمل) validation for Cash vs Credit entities</t>
+          <t>Medicines tab credit percentage field (نسبة التحمل) locked/readonly for Cash entity</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>فيلد نسبة التحمل في تاب صرف الأدوية (مغلق للجهات النقدي ومفتوح للجهات الآجل من 0 لـ 100%)</t>
+          <t>فيلد نسبة التحمل في تاب صرف الأدوية (مغلق ومحمي للجهات النقدي)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Verify credit percentage field is locked/readonly for cash entity visits and open/editable (0-100%) for credit entity visits ('اليكو').</t>
+          <t>Verify credit percentage field is locked/readonly for cash entity visits.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>التحقق من أن فيلد نسبة التحمل يكون مغلقاً في حالة جهة المريض نقدي، ومفتوحاً ويقبل نسب من 0 إلى 100% في حالة جهة المريض آجل.</t>
+          <t>التحقق من أن فيلد نسبة التحمل يكون مغلقاً وغير قابل للتعديل في حالة جهة المريض نقدي.</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5486,7 +5485,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>medicinesTabCreditPctFieldValidationCashVsCredit</t>
+          <t>medicinesTabCreditPctReadonlyForCashEntity</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5502,6 +5501,78 @@
       <c r="N65" t="inlineStr">
         <is>
           <t>Added 2026-08-19 — Medicines tab credit percentage field cash vs credit validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TC-OPD-029</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Outpatient Visits (OPD Clinics)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>العيادات الخارجية</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Medicines tab credit percentage field (نسبة التحمل) enabled/editable (0-100%) for Credit entity</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>فيلد نسبة التحمل في تاب صرف الأدوية (مفتوح وقابل لإدخال 0-100% للجهات الآجل)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Verify credit percentage field is enabled and editable (0-100%) for credit entity visits ('اليكو').</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>التحقق من أن فيلد نسبة التحمل يكون مفتوحاً ويقبل نسب من 0 إلى 100% في حالة جهة المريض آجل ('اليكو').</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>medicinesTabCreditPctEditableForCreditEntity</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>OutpatientCycleTests</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Added 2026-08-19 — Medicines tab credit percentage field credit entity validation</t>
         </is>
       </c>
     </row>
@@ -5607,10 +5678,10 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>28</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>27</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0</v>

</xml_diff>